<commit_message>
fix: tambahkan judul paper lengkap di tabel voting sheet 2
</commit_message>
<xml_diff>
--- a/rekap_dataset_biner_dan_irisan improve.xlsx
+++ b/rekap_dataset_biner_dan_irisan improve.xlsx
@@ -953,12 +953,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -967,6 +967,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1389,7 +1390,8 @@
       <c r="H21" s="7" t="n"/>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="7" t="n"/>
-      <c r="K21" s="8" t="n"/>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1399,56 +1401,61 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
+          <t>Judul Paper</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
           <t>Jurnal &amp; Tahun</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>NV</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>BKL</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>DF</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>VASC</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>BCC</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>AKIEC</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>SCC</t>
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Kousis et al.</t>
@@ -1456,113 +1463,123 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>Deep Learning Methods for Accurate Skin Cancer Recognition and Mobile Application</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
           <t>Electronics (MDPI), 2022</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="H23" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="I23" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="J23" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J23" s="15" t="inlineStr">
+      <c r="K23" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Ghosh et al. (SkinNet-16)</t>
+          <t>Ghosh et al.</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
+          <t>SkinNet-16: A deep learning approach to identify benign and malignant skin lesions</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
           <t>Frontiers in Oncology, 2022</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="F24" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H24" s="15" t="inlineStr">
+      <c r="I24" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I24" s="15" t="inlineStr">
+      <c r="J24" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J24" s="15" t="inlineStr">
+      <c r="K24" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr">
+      <c r="L24" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Harangi et al.</t>
@@ -1570,56 +1587,61 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
+          <t>Assisted deep learning framework for multi-class skin lesion classification considering a binary classification support</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
           <t>Biomedical Signal Proc. &amp; Control (Elsevier), 2020</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>HAM10000 / 2018</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G25" s="15" t="inlineStr">
+      <c r="H25" s="15" t="inlineStr">
         <is>
           <t>Ganas*</t>
         </is>
       </c>
-      <c r="H25" s="15" t="inlineStr">
+      <c r="I25" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I25" s="15" t="inlineStr">
+      <c r="J25" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J25" s="15" t="inlineStr">
+      <c r="K25" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="36" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Ameri</t>
@@ -1627,56 +1649,61 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
+          <t>A deep learning approach to skin cancer detection in dermoscopy images</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
           <t>J. Biomed. Physics &amp; Eng. (JBPE), 2020</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="F26" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F26" s="12" t="inlineStr">
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>Exclude</t>
         </is>
       </c>
-      <c r="H26" s="15" t="inlineStr">
+      <c r="I26" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I26" s="15" t="inlineStr">
+      <c r="J26" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J26" s="15" t="inlineStr">
+      <c r="K26" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr">
+      <c r="L26" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Barata et al.</t>
@@ -1684,56 +1711,61 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
+          <t>Explainable skin lesion diagnosis using taxonomies</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
           <t>Pattern Recognition (Elsevier), 2020</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>ISIC 2017</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H27" s="15" t="inlineStr">
+      <c r="I27" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="L27" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Jojoa Acosta et al.</t>
@@ -1741,113 +1773,123 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
+          <t>Melanoma diagnosis using deep learning techniques on dermatoscopic images</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
           <t>BMC Medical Imaging (Springer), 2021</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>ISIC 2017</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H28" s="15" t="inlineStr">
+      <c r="I28" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="K28" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="L28" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="36" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Yao et al. (MorphoNet)</t>
+          <t>Yao et al.</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>MorphoNet: An Interpretable Hierarchical Deep Learning Framework for Multi-Class Skin Lesion Classification</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
           <t>Bioengineering (MDPI), 2026</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>HAM10k &amp; 2019</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="H29" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H29" s="15" t="inlineStr">
+      <c r="I29" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I29" s="15" t="inlineStr">
+      <c r="J29" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J29" s="15" t="inlineStr">
+      <c r="K29" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K29" s="15" t="inlineStr">
+      <c r="L29" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="36" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Venugopal et al.</t>
@@ -1855,50 +1897,55 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>Multiclass skin cancer classification using ensemble of fine-tuned deep learning models</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
           <t>Data Analysis Journal (Elsevier), 2023</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>ISIC 2019</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G30" s="12" t="inlineStr">
+      <c r="H30" s="12" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H30" s="15" t="inlineStr">
+      <c r="I30" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="I30" s="15" t="inlineStr">
+      <c r="J30" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J30" s="15" t="inlineStr">
+      <c r="K30" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K30" s="15" t="inlineStr">
+      <c r="L30" s="15" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
@@ -1910,52 +1957,53 @@
           <t>KONSENSUS (VOTING)</t>
         </is>
       </c>
-      <c r="B31" s="26" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr"/>
+      <c r="C31" s="26" t="inlineStr">
         <is>
           <t>Mayoritas Literatur</t>
         </is>
       </c>
-      <c r="C31" s="26" t="inlineStr">
+      <c r="D31" s="26" t="inlineStr">
         <is>
           <t>Semua Sumber</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>JINAK (100%)</t>
         </is>
       </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>JINAK (100%)</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr">
+      <c r="G31" s="12" t="inlineStr">
         <is>
           <t>JINAK (100%)</t>
         </is>
       </c>
-      <c r="G31" s="12" t="inlineStr">
+      <c r="H31" s="12" t="inlineStr">
         <is>
           <t>JINAK (80%)</t>
         </is>
       </c>
-      <c r="H31" s="15" t="inlineStr">
+      <c r="I31" s="15" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
       </c>
-      <c r="I31" s="15" t="inlineStr">
+      <c r="J31" s="15" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
       </c>
-      <c r="J31" s="15" t="inlineStr">
+      <c r="K31" s="15" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
       </c>
-      <c r="K31" s="15" t="inlineStr">
+      <c r="L31" s="15" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
@@ -1964,10 +2012,10 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A21:K21"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A21:L21"/>
     <mergeCell ref="A16:G19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
style: ubah tampilan tabel jadi bersih kayak buatan manusia - border hitam, bg putih, grid lines on, font highlight saja
</commit_message>
<xml_diff>
--- a/rekap_dataset_biner_dan_irisan improve.xlsx
+++ b/rekap_dataset_biner_dan_irisan improve.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,60 +31,54 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002D3436"/>
-      <sz val="13"/>
+      <color rgb="00000000"/>
+      <sz val="14"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00636E72"/>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00444444"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="002D3436"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="002D3436"/>
+      <color rgb="001A7A2E"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="00636E72"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002D3436"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="0027AE60"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00E74C3C"/>
-      <sz val="10"/>
+      <color rgb="00C0392B"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -93,47 +87,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002C3E50"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EBF0F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F8F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDEDEC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8EDF2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5F5E3"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -147,23 +111,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -171,10 +135,10 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -183,29 +147,29 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </left>
       <right/>
       <top/>
@@ -215,7 +179,7 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </right>
       <top/>
       <bottom/>
@@ -223,12 +187,12 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </left>
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -237,18 +201,18 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="00D5D8DC"/>
+        <color rgb="00000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -256,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -267,45 +231,27 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -315,29 +261,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -701,7 +644,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002C3E50"/>
+    <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -773,22 +716,22 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Dataset yang dipakai</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>HAM10000 + ISIC 2019 + ISIC 2017 (semua partisi)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>HAM10000 + ISIC 2019 Train + ISIC 2017 (Train/Val/Test)</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Keduanya pakai 3 sumber dataset yang sama</t>
         </is>
@@ -817,22 +760,22 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Jumlah kelas</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>2 kelas: Benign (0) dan Malignant (1)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>3 kelas: NV (0), MEL (1), BKL (2)</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Biner pakai semua 8 jenis penyakit, irisan cuma 3</t>
         </is>
@@ -861,76 +804,76 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Acuan paper utama</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Konsensus voting 8 paper internasional (Elsevier, MDPI, Springer, Frontiers)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Tschandl et al. (Nature 2018), Codella et al. (IEEE ISBI 2018), Baig (2023), Ichim (2023)</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Semua pemetaan didasarkan rujukan jurnal bereputasi (Scopus Q1 / Nature)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Catatan Penting untuk Dosen Pembimbing</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="8" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="7" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>1. Konsistensi data: Seluruh 22.051 citra irisan berada di dalam dataset biner (33.552). Tidak ada satu pun gambar yang bentrok labelnya.</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="8" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>2. Validitas label BKL: Penggabungan 'Seborrheic Keratosis' (ISIC 2017) ke 'BKL' sudah sesuai standar Nature Scientific Data (Tschandl et al., 2018, hal. 7).</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="8" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="7" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>3. Data siap modeling: Dataset irisan 3 kelas sudah dipartisi Train (17.656) / Val (2.192) / Test (2.203) dengan jaminan 0% kebocoran lesi pasien.</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="8" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>4. Pipeline lengkap: Seluruh kode Data Understanding, Data Preparation, sampai skrip training PyTorch (ResNet-50 &amp; EfficientNet-B0) sudah terstruktur dan terverifikasi.</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="8" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -949,7 +892,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002980B9"/>
+    <tabColor rgb="005B9BD5"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -985,17 +928,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>A. Kode Harmonisasi 8 Kelas Diagnosis Kulit</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1035,44 +978,44 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>NV</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Melanocytic Nevus (tahi lalat jinak)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>nv</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>NV</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>nevus</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Benign (0)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>MEL</t>
         </is>
@@ -1097,56 +1040,56 @@
           <t>melanoma</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Malignant (1)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>BKL</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Benign Keratosis (keratosis seboroik)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>bkl</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>BKL</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>seborrheic_keratosis</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Benign (0)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>BCC</t>
         </is>
@@ -1171,56 +1114,56 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>Malignant (1)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>AKIEC</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Actinic Keratosis (pre-kanker)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>akiec</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>AK</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>Pre-kanker/Ganas</t>
         </is>
       </c>
-      <c r="G10" s="15" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>Malignant (1)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>SCC</t>
         </is>
@@ -1245,56 +1188,56 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Malignant (1)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>VASC</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Vascular Lesion (lesi pembuluh darah)</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>vasc</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>VASC</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>Benign (0)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>DF</t>
         </is>
@@ -1319,79 +1262,79 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
         <is>
           <t>Benign (0)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>B. Kenapa 'Seborrheic Keratosis' (ISIC 2017) Digabung ke 'BKL'</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="8" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Tschandl, Rosendahl, &amp; Kittler (2018) di Nature Scientific Data, hal. 7, menjelaskan:
 "Benign keratosis is a generic class that includes seborrheic keratoses (senile wart), solar lentigo, and lichen-planus like keratoses (LPLK)... we grouped them together because they are similar biologically and often reported under the same generic term histopathologically."
 Jadi penggabungan ini bukan keputusan kita sendiri -- ini standar resmi dari konsorsium ISIC sejak 2018.</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="19" t="n"/>
-      <c r="F16" s="19" t="n"/>
-      <c r="G16" s="20" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="n"/>
-      <c r="G17" s="22" t="n"/>
+      <c r="A17" s="15" t="n"/>
+      <c r="G17" s="16" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="n"/>
-      <c r="G18" s="22" t="n"/>
+      <c r="A18" s="15" t="n"/>
+      <c r="G18" s="16" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="25" t="n"/>
+      <c r="A19" s="17" t="n"/>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="19" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>C. Matriks Voting 8 Paper Internasional (Pemetaan Biner)</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="8" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1476,37 +1419,37 @@
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H23" s="12" t="inlineStr">
+      <c r="H23" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="I23" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J23" s="15" t="inlineStr">
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K23" s="15" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
@@ -1518,62 +1461,62 @@
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Ghosh et al.</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>SkinNet-16: A deep learning approach to identify benign and malignant skin lesions</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Frontiers in Oncology, 2022</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="G24" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="H24" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="I24" s="15" t="inlineStr">
+      <c r="I24" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J24" s="15" t="inlineStr">
+      <c r="J24" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K24" s="15" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="L24" s="5" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1600,37 +1543,37 @@
           <t>HAM10000 / 2018</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G25" s="12" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H25" s="15" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>Ganas*</t>
         </is>
       </c>
-      <c r="I25" s="15" t="inlineStr">
+      <c r="I25" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J25" s="15" t="inlineStr">
+      <c r="J25" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K25" s="15" t="inlineStr">
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
@@ -1642,62 +1585,62 @@
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Ameri</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>A deep learning approach to skin cancer detection in dermoscopy images</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>J. Biomed. Physics &amp; Eng. (JBPE), 2020</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F26" s="12" t="inlineStr">
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G26" s="12" t="inlineStr">
+      <c r="G26" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Exclude</t>
         </is>
       </c>
-      <c r="I26" s="15" t="inlineStr">
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J26" s="15" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K26" s="15" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1724,12 +1667,12 @@
           <t>ISIC 2017</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
@@ -1744,7 +1687,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I27" s="15" t="inlineStr">
+      <c r="I27" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
@@ -1766,62 +1709,62 @@
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Jojoa Acosta et al.</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Melanoma diagnosis using deep learning techniques on dermatoscopic images</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>BMC Medical Imaging (Springer), 2021</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>ISIC 2017</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I28" s="15" t="inlineStr">
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L28" s="5" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1848,162 +1791,162 @@
           <t>HAM10k &amp; 2019</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="F29" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="G29" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H29" s="12" t="inlineStr">
+      <c r="H29" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="I29" s="15" t="inlineStr">
+      <c r="I29" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J29" s="15" t="inlineStr">
+      <c r="J29" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K29" s="15" t="inlineStr">
+      <c r="K29" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="L29" s="15" t="inlineStr">
+      <c r="L29" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Venugopal et al.</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Multiclass skin cancer classification using ensemble of fine-tuned deep learning models</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Data Analysis Journal (Elsevier), 2023</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>ISIC 2019</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="F30" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="G30" s="12" t="inlineStr">
+      <c r="G30" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="H30" s="12" t="inlineStr">
+      <c r="H30" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="I30" s="15" t="inlineStr">
+      <c r="I30" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="J30" s="15" t="inlineStr">
+      <c r="J30" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="K30" s="15" t="inlineStr">
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="L30" s="15" t="inlineStr">
+      <c r="L30" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="26" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>KONSENSUS (VOTING)</t>
         </is>
       </c>
-      <c r="B31" s="26" t="inlineStr"/>
-      <c r="C31" s="26" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr"/>
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>Mayoritas Literatur</t>
         </is>
       </c>
-      <c r="D31" s="26" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>Semua Sumber</t>
         </is>
       </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>JINAK (100%)</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr">
+      <c r="F31" s="21" t="inlineStr">
         <is>
           <t>JINAK (100%)</t>
         </is>
       </c>
-      <c r="G31" s="12" t="inlineStr">
+      <c r="G31" s="21" t="inlineStr">
         <is>
           <t>JINAK (100%)</t>
         </is>
       </c>
-      <c r="H31" s="12" t="inlineStr">
+      <c r="H31" s="21" t="inlineStr">
         <is>
           <t>JINAK (80%)</t>
         </is>
       </c>
-      <c r="I31" s="15" t="inlineStr">
+      <c r="I31" s="22" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
       </c>
-      <c r="J31" s="15" t="inlineStr">
+      <c r="J31" s="22" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
       </c>
-      <c r="K31" s="15" t="inlineStr">
+      <c r="K31" s="22" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
       </c>
-      <c r="L31" s="15" t="inlineStr">
+      <c r="L31" s="22" t="inlineStr">
         <is>
           <t>GANAS (100%)</t>
         </is>
@@ -2025,7 +1968,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="008E44AD"/>
+    <tabColor rgb="00A5A5A5"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2060,17 +2003,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>A. Proses Deduplikasi Antar-Dataset</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2110,29 +2053,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Part 1 &amp; 2</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="23" t="n">
         <v>10015</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="23" t="n">
         <v>10015</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="24" t="n">
         <v>0.2985</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Dipertahankan 100% utuh, tidak ada yang dibuang</t>
         </is>
@@ -2149,16 +2092,16 @@
           <t>Training Input</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="23" t="n">
         <v>25331</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="23" t="n">
         <v>10015</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="23" t="n">
         <v>15316</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="24" t="n">
         <v>0.4565</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -2168,29 +2111,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>ISIC 2019</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Test Input</t>
         </is>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="23" t="n">
         <v>8238</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="23" t="n">
         <v>2047</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="23" t="n">
         <v>6191</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="24" t="n">
         <v>0.1845</v>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>2.047 citra UNK (out-of-distribution) dibuang</t>
         </is>
@@ -2207,16 +2150,16 @@
           <t>Training Data</t>
         </is>
       </c>
-      <c r="C9" s="29" t="n">
+      <c r="C9" s="23" t="n">
         <v>2000</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="23" t="n">
         <v>717</v>
       </c>
-      <c r="E9" s="29" t="n">
+      <c r="E9" s="23" t="n">
         <v>1283</v>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="F9" s="24" t="n">
         <v>0.0382</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -2226,29 +2169,29 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>ISIC 2017</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="23" t="n">
         <v>600</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="23" t="n">
         <v>599</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="24" t="n">
         <v>0.0179</v>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>1 duplikat dibuang</t>
         </is>
@@ -2265,16 +2208,16 @@
           <t>Validation Data</t>
         </is>
       </c>
-      <c r="C11" s="29" t="n">
+      <c r="C11" s="23" t="n">
         <v>150</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="29" t="n">
+      <c r="E11" s="23" t="n">
         <v>148</v>
       </c>
-      <c r="F11" s="30" t="n">
+      <c r="F11" s="24" t="n">
         <v>0.0044</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -2284,50 +2227,50 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>6 Partisi</t>
         </is>
       </c>
-      <c r="C12" s="31" t="n">
+      <c r="C12" s="25" t="n">
         <v>46334</v>
       </c>
-      <c r="D12" s="31" t="n">
+      <c r="D12" s="25" t="n">
         <v>12782</v>
       </c>
-      <c r="E12" s="31" t="n">
+      <c r="E12" s="25" t="n">
         <v>33552</v>
       </c>
-      <c r="F12" s="32" t="n">
+      <c r="F12" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="26" t="inlineStr">
+      <c r="G12" s="20" t="inlineStr">
         <is>
           <t>33.552 citra berlabel bersih, 100% unik</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>B. Sebaran 8 Kelas Diagnosis per Sumber Dataset</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
-      <c r="K14" s="8" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2387,48 +2330,48 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>NV</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Melanocytic Nevus</t>
         </is>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="23" t="n">
         <v>6705</v>
       </c>
-      <c r="D16" s="27" t="n">
+      <c r="D16" s="23" t="n">
         <v>6170</v>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="23" t="n">
         <v>2495</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="23" t="n">
         <v>804</v>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="23" t="n">
         <v>393</v>
       </c>
-      <c r="H16" s="27" t="n">
+      <c r="H16" s="23" t="n">
         <v>76</v>
       </c>
-      <c r="I16" s="27" t="n">
+      <c r="I16" s="23" t="n">
         <v>16643</v>
       </c>
-      <c r="J16" s="28" t="n">
+      <c r="J16" s="24" t="n">
         <v>0.496</v>
       </c>
-      <c r="K16" s="11" t="inlineStr">
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>MEL</t>
         </is>
@@ -2438,79 +2381,79 @@
           <t>Melanoma</t>
         </is>
       </c>
-      <c r="C17" s="29" t="n">
+      <c r="C17" s="23" t="n">
         <v>1113</v>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D17" s="23" t="n">
         <v>3409</v>
       </c>
-      <c r="E17" s="29" t="n">
+      <c r="E17" s="23" t="n">
         <v>1327</v>
       </c>
-      <c r="F17" s="29" t="n">
+      <c r="F17" s="23" t="n">
         <v>227</v>
       </c>
-      <c r="G17" s="29" t="n">
+      <c r="G17" s="23" t="n">
         <v>116</v>
       </c>
-      <c r="H17" s="29" t="n">
+      <c r="H17" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="I17" s="29" t="n">
+      <c r="I17" s="23" t="n">
         <v>6222</v>
       </c>
-      <c r="J17" s="30" t="n">
+      <c r="J17" s="24" t="n">
         <v>0.1854</v>
       </c>
-      <c r="K17" s="14" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>BCC</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Basal Cell Carcinoma</t>
         </is>
       </c>
-      <c r="C18" s="27" t="n">
+      <c r="C18" s="23" t="n">
         <v>514</v>
       </c>
-      <c r="D18" s="27" t="n">
+      <c r="D18" s="23" t="n">
         <v>2809</v>
       </c>
-      <c r="E18" s="27" t="n">
+      <c r="E18" s="23" t="n">
         <v>975</v>
       </c>
-      <c r="F18" s="27" t="n">
+      <c r="F18" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="27" t="n">
+      <c r="G18" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="27" t="n">
+      <c r="H18" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="27" t="n">
+      <c r="I18" s="23" t="n">
         <v>4298</v>
       </c>
-      <c r="J18" s="28" t="n">
+      <c r="J18" s="24" t="n">
         <v>0.1281</v>
       </c>
-      <c r="K18" s="16" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>BKL</t>
         </is>
@@ -2520,79 +2463,79 @@
           <t>Benign Keratosis</t>
         </is>
       </c>
-      <c r="C19" s="29" t="n">
+      <c r="C19" s="23" t="n">
         <v>1099</v>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="23" t="n">
         <v>1525</v>
       </c>
-      <c r="E19" s="29" t="n">
+      <c r="E19" s="23" t="n">
         <v>660</v>
       </c>
-      <c r="F19" s="29" t="n">
+      <c r="F19" s="23" t="n">
         <v>252</v>
       </c>
-      <c r="G19" s="29" t="n">
+      <c r="G19" s="23" t="n">
         <v>90</v>
       </c>
-      <c r="H19" s="29" t="n">
+      <c r="H19" s="23" t="n">
         <v>42</v>
       </c>
-      <c r="I19" s="29" t="n">
+      <c r="I19" s="23" t="n">
         <v>3668</v>
       </c>
-      <c r="J19" s="30" t="n">
+      <c r="J19" s="24" t="n">
         <v>0.1093</v>
       </c>
-      <c r="K19" s="17" t="inlineStr">
+      <c r="K19" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>AKIEC</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Actinic Keratosis</t>
         </is>
       </c>
-      <c r="C20" s="27" t="n">
+      <c r="C20" s="23" t="n">
         <v>327</v>
       </c>
-      <c r="D20" s="27" t="n">
+      <c r="D20" s="23" t="n">
         <v>737</v>
       </c>
-      <c r="E20" s="27" t="n">
+      <c r="E20" s="23" t="n">
         <v>374</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="27" t="n">
+      <c r="G20" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="27" t="n">
+      <c r="H20" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="27" t="n">
+      <c r="I20" s="23" t="n">
         <v>1438</v>
       </c>
-      <c r="J20" s="28" t="n">
+      <c r="J20" s="24" t="n">
         <v>0.0429</v>
       </c>
-      <c r="K20" s="16" t="inlineStr">
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>Pre-kanker/Ganas</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>SCC</t>
         </is>
@@ -2602,79 +2545,79 @@
           <t>Squamous Cell Carcinoma</t>
         </is>
       </c>
-      <c r="C21" s="29" t="n">
+      <c r="C21" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D21" s="29" t="n">
+      <c r="D21" s="23" t="n">
         <v>431</v>
       </c>
-      <c r="E21" s="29" t="n">
+      <c r="E21" s="23" t="n">
         <v>165</v>
       </c>
-      <c r="F21" s="29" t="n">
+      <c r="F21" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="29" t="n">
+      <c r="G21" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="29" t="n">
+      <c r="H21" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="29" t="n">
+      <c r="I21" s="23" t="n">
         <v>596</v>
       </c>
-      <c r="J21" s="30" t="n">
+      <c r="J21" s="24" t="n">
         <v>0.0178</v>
       </c>
-      <c r="K21" s="14" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>VASC</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Vascular Lesion</t>
         </is>
       </c>
-      <c r="C22" s="27" t="n">
+      <c r="C22" s="23" t="n">
         <v>142</v>
       </c>
-      <c r="D22" s="27" t="n">
+      <c r="D22" s="23" t="n">
         <v>111</v>
       </c>
-      <c r="E22" s="27" t="n">
+      <c r="E22" s="23" t="n">
         <v>104</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="27" t="n">
+      <c r="I22" s="23" t="n">
         <v>357</v>
       </c>
-      <c r="J22" s="28" t="n">
+      <c r="J22" s="24" t="n">
         <v>0.0106</v>
       </c>
-      <c r="K22" s="11" t="inlineStr">
+      <c r="K22" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>DF</t>
         </is>
@@ -2684,84 +2627,84 @@
           <t>Dermatofibroma</t>
         </is>
       </c>
-      <c r="C23" s="29" t="n">
+      <c r="C23" s="23" t="n">
         <v>115</v>
       </c>
-      <c r="D23" s="29" t="n">
+      <c r="D23" s="23" t="n">
         <v>124</v>
       </c>
-      <c r="E23" s="29" t="n">
+      <c r="E23" s="23" t="n">
         <v>91</v>
       </c>
-      <c r="F23" s="29" t="n">
+      <c r="F23" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="29" t="n">
+      <c r="G23" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="29" t="n">
+      <c r="H23" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="I23" s="29" t="n">
+      <c r="I23" s="23" t="n">
         <v>330</v>
       </c>
-      <c r="J23" s="30" t="n">
+      <c r="J23" s="24" t="n">
         <v>0.0098</v>
       </c>
-      <c r="K23" s="17" t="inlineStr">
+      <c r="K23" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="26" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>8 Kelas</t>
         </is>
       </c>
-      <c r="C24" s="31" t="n">
+      <c r="C24" s="25" t="n">
         <v>10015</v>
       </c>
-      <c r="D24" s="31" t="n">
+      <c r="D24" s="25" t="n">
         <v>15316</v>
       </c>
-      <c r="E24" s="31" t="n">
+      <c r="E24" s="25" t="n">
         <v>6191</v>
       </c>
-      <c r="F24" s="31" t="n">
+      <c r="F24" s="25" t="n">
         <v>1283</v>
       </c>
-      <c r="G24" s="31" t="n">
+      <c r="G24" s="25" t="n">
         <v>599</v>
       </c>
-      <c r="H24" s="31" t="n">
+      <c r="H24" s="25" t="n">
         <v>148</v>
       </c>
-      <c r="I24" s="31" t="n">
+      <c r="I24" s="25" t="n">
         <v>33552</v>
       </c>
-      <c r="J24" s="32" t="n">
+      <c r="J24" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="K24" s="26" t="inlineStr"/>
+      <c r="K24" s="20" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>C. Distribusi Target Akhir (Benign vs Malignant)</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="8" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -2796,36 +2739,36 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="n">
+      <c r="A28" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Benign (Jinak)</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>NV (16.643) + BKL (3.668) + VASC (357) + DF (330)</t>
         </is>
       </c>
-      <c r="D28" s="27" t="n">
+      <c r="D28" s="23" t="n">
         <v>20998</v>
       </c>
-      <c r="E28" s="28" t="n">
+      <c r="E28" s="24" t="n">
         <v>0.6258</v>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>1,67 : 1 (mayoritas)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="29" t="n">
+      <c r="A29" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Malignant (Ganas)</t>
         </is>
@@ -2835,10 +2778,10 @@
           <t>MEL (6.222) + BCC (4.298) + AKIEC (1.438) + SCC (596)</t>
         </is>
       </c>
-      <c r="D29" s="29" t="n">
+      <c r="D29" s="23" t="n">
         <v>12554</v>
       </c>
-      <c r="E29" s="30" t="n">
+      <c r="E29" s="24" t="n">
         <v>0.3742</v>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -2848,28 +2791,28 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="26" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="B30" s="26" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C30" s="26" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>8 Kelas Gabungan</t>
         </is>
       </c>
-      <c r="D30" s="31" t="n">
+      <c r="D30" s="25" t="n">
         <v>33552</v>
       </c>
-      <c r="E30" s="32" t="n">
+      <c r="E30" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F30" s="26" t="inlineStr">
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>Siap Modeling</t>
         </is>
@@ -2890,7 +2833,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0027AE60"/>
+    <tabColor rgb="0070AD47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2923,17 +2866,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>A. Sebaran 3 Kelas per Sumber Dataset</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2973,29 +2916,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Part 1 &amp; 2 (100% utuh)</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="23" t="n">
         <v>6705</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="23" t="n">
         <v>1113</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="23" t="n">
         <v>1099</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="23" t="n">
         <v>8917</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="24" t="n">
         <v>0.4044</v>
       </c>
     </row>
@@ -3010,46 +2953,46 @@
           <t>Training (non-HAM)</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="23" t="n">
         <v>6170</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="23" t="n">
         <v>3409</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="23" t="n">
         <v>1525</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="23" t="n">
         <v>11104</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="24" t="n">
         <v>0.5036</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>ISIC 2017</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Training Data</t>
         </is>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="23" t="n">
         <v>804</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="23" t="n">
         <v>227</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="23" t="n">
         <v>252</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="23" t="n">
         <v>1283</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="24" t="n">
         <v>0.0582</v>
       </c>
     </row>
@@ -3064,88 +3007,88 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="C9" s="29" t="n">
+      <c r="C9" s="23" t="n">
         <v>393</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="23" t="n">
         <v>116</v>
       </c>
-      <c r="E9" s="29" t="n">
+      <c r="E9" s="23" t="n">
         <v>90</v>
       </c>
-      <c r="F9" s="29" t="n">
+      <c r="F9" s="23" t="n">
         <v>599</v>
       </c>
-      <c r="G9" s="30" t="n">
+      <c r="G9" s="24" t="n">
         <v>0.0272</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>ISIC 2017</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Validation Data</t>
         </is>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="23" t="n">
         <v>76</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="23" t="n">
         <v>42</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="23" t="n">
         <v>148</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="24" t="n">
         <v>0.0067</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>3 Dataset</t>
         </is>
       </c>
-      <c r="C11" s="31" t="n">
+      <c r="C11" s="25" t="n">
         <v>14148</v>
       </c>
-      <c r="D11" s="31" t="n">
+      <c r="D11" s="25" t="n">
         <v>4895</v>
       </c>
-      <c r="E11" s="31" t="n">
+      <c r="E11" s="25" t="n">
         <v>3008</v>
       </c>
-      <c r="F11" s="31" t="n">
+      <c r="F11" s="25" t="n">
         <v>22051</v>
       </c>
-      <c r="G11" s="32" t="n">
+      <c r="G11" s="26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>B. Ringkasan 3 Kelas Harmonisasi</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="8" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3185,10 +3128,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="n">
+      <c r="A15" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>NV</t>
         </is>
@@ -3198,15 +3141,15 @@
           <t>Melanocytic Nevus (tahi lalat jinak)</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E15" s="29" t="n">
+      <c r="E15" s="23" t="n">
         <v>14148</v>
       </c>
-      <c r="F15" s="30" t="n">
+      <c r="F15" s="24" t="n">
         <v>0.6415999999999999</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -3216,41 +3159,41 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="n">
+      <c r="A16" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>MEL</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Melanoma (kanker kulit ganas)</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Ganas</t>
         </is>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="23" t="n">
         <v>4895</v>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="24" t="n">
         <v>0.222</v>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>1.50 (perhatian klinis utama)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="n">
+      <c r="A17" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>BKL</t>
         </is>
@@ -3260,15 +3203,15 @@
           <t>Benign Keratosis (keratosis seboroik)</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Jinak</t>
         </is>
       </c>
-      <c r="E17" s="29" t="n">
+      <c r="E17" s="23" t="n">
         <v>3008</v>
       </c>
-      <c r="F17" s="30" t="n">
+      <c r="F17" s="24" t="n">
         <v>0.1364</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -3278,19 +3221,19 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>C. Partisi Data (Lesion-Aware Split 80:10:10)</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="8" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -3350,19 +3293,19 @@
           <t>80%</t>
         </is>
       </c>
-      <c r="C21" s="29" t="n">
+      <c r="C21" s="23" t="n">
         <v>17656</v>
       </c>
-      <c r="D21" s="30" t="n">
+      <c r="D21" s="24" t="n">
         <v>0.8007</v>
       </c>
-      <c r="E21" s="29" t="n">
+      <c r="E21" s="23" t="n">
         <v>11302</v>
       </c>
-      <c r="F21" s="29" t="n">
+      <c r="F21" s="23" t="n">
         <v>3902</v>
       </c>
-      <c r="G21" s="29" t="n">
+      <c r="G21" s="23" t="n">
         <v>2452</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -3370,44 +3313,44 @@
           <t>0 overlap</t>
         </is>
       </c>
-      <c r="I21" s="33" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Bebas Kebocoran</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C22" s="27" t="n">
+      <c r="C22" s="23" t="n">
         <v>2192</v>
       </c>
-      <c r="D22" s="28" t="n">
+      <c r="D22" s="24" t="n">
         <v>0.0994</v>
       </c>
-      <c r="E22" s="27" t="n">
+      <c r="E22" s="23" t="n">
         <v>1455</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="23" t="n">
         <v>450</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="23" t="n">
         <v>287</v>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>0 overlap</t>
         </is>
       </c>
-      <c r="I22" s="33" t="inlineStr">
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>Bebas Kebocoran</t>
         </is>
@@ -3424,19 +3367,19 @@
           <t>10%</t>
         </is>
       </c>
-      <c r="C23" s="29" t="n">
+      <c r="C23" s="23" t="n">
         <v>2203</v>
       </c>
-      <c r="D23" s="30" t="n">
+      <c r="D23" s="24" t="n">
         <v>0.0999</v>
       </c>
-      <c r="E23" s="29" t="n">
+      <c r="E23" s="23" t="n">
         <v>1391</v>
       </c>
-      <c r="F23" s="29" t="n">
+      <c r="F23" s="23" t="n">
         <v>543</v>
       </c>
-      <c r="G23" s="29" t="n">
+      <c r="G23" s="23" t="n">
         <v>269</v>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -3444,44 +3387,44 @@
           <t>0 overlap</t>
         </is>
       </c>
-      <c r="I23" s="33" t="inlineStr">
+      <c r="I23" s="10" t="inlineStr">
         <is>
           <t>Bebas Kebocoran</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="26" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="C24" s="31" t="n">
+      <c r="C24" s="25" t="n">
         <v>22051</v>
       </c>
-      <c r="D24" s="32" t="n">
+      <c r="D24" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="31" t="n">
+      <c r="E24" s="25" t="n">
         <v>14148</v>
       </c>
-      <c r="F24" s="31" t="n">
+      <c r="F24" s="25" t="n">
         <v>4895</v>
       </c>
-      <c r="G24" s="31" t="n">
+      <c r="G24" s="25" t="n">
         <v>3008</v>
       </c>
-      <c r="H24" s="26" t="inlineStr">
+      <c r="H24" s="20" t="inlineStr">
         <is>
           <t>0 overlap</t>
         </is>
       </c>
-      <c r="I24" s="26" t="inlineStr">
+      <c r="I24" s="20" t="inlineStr">
         <is>
           <t>Lolos Semua</t>
         </is>
@@ -3502,7 +3445,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00E67E22"/>
+    <tabColor rgb="00ED7D31"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3537,15 +3480,15 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>A. Hasil Audit Komputasional</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="8" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3575,27 +3518,27 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Kesesuaian ID citra (irisan ada di biner)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>22.051 dari 22.051 (100%)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>100% harus ada</t>
         </is>
       </c>
-      <c r="D6" s="33" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>LOLOS</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Semua gambar irisan ada di dalam dataset biner</t>
         </is>
@@ -3617,7 +3560,7 @@
           <t>0 mismatch</t>
         </is>
       </c>
-      <c r="D7" s="33" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>LOLOS</t>
         </is>
@@ -3629,27 +3572,27 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Ketidakcocokan sumber (source mismatch)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>0 kasus (0%)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>0 mismatch</t>
         </is>
       </c>
-      <c r="D8" s="33" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>LOLOS</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Asal dataset (HAM10k, 2019, 2017) 100% konsisten</t>
         </is>
@@ -3671,7 +3614,7 @@
           <t>100% ada</t>
         </is>
       </c>
-      <c r="D9" s="33" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>LOLOS</t>
         </is>
@@ -3683,27 +3626,27 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Kebocoran lesi antar-subset</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>0 lesi tumpang tindih</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>0 overlap</t>
         </is>
       </c>
-      <c r="D10" s="33" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>LOLOS</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>StratifiedGroupKFold menjamin tidak ada pasien bocor antar Train/Val/Test</t>
         </is>
@@ -3725,7 +3668,7 @@
           <t>0 NaN</t>
         </is>
       </c>
-      <c r="D11" s="33" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>LOLOS</t>
         </is>
@@ -3737,21 +3680,21 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>B. Rincian 11.501 Citra yang Tidak Masuk Irisan (Kenapa?)</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
-      <c r="K13" s="8" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3816,31 +3759,31 @@
           <t>HAM10000</t>
         </is>
       </c>
-      <c r="B15" s="29" t="n">
+      <c r="B15" s="23" t="n">
         <v>327</v>
       </c>
-      <c r="C15" s="29" t="n">
+      <c r="C15" s="23" t="n">
         <v>514</v>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="29" t="n">
+      <c r="E15" s="23" t="n">
         <v>115</v>
       </c>
-      <c r="F15" s="29" t="n">
+      <c r="F15" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="29" t="n">
+      <c r="G15" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="29" t="n">
+      <c r="H15" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="29" t="n">
+      <c r="I15" s="23" t="n">
         <v>142</v>
       </c>
-      <c r="J15" s="29" t="n">
+      <c r="J15" s="23" t="n">
         <v>1098</v>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -3850,39 +3793,39 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ISIC 2019 Training</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
+      <c r="B16" s="23" t="n">
         <v>737</v>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="23" t="n">
         <v>2809</v>
       </c>
-      <c r="D16" s="27" t="n">
+      <c r="D16" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="23" t="n">
         <v>124</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="27" t="n">
+      <c r="H16" s="23" t="n">
         <v>431</v>
       </c>
-      <c r="I16" s="27" t="n">
+      <c r="I16" s="23" t="n">
         <v>111</v>
       </c>
-      <c r="J16" s="27" t="n">
+      <c r="J16" s="23" t="n">
         <v>4212</v>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Kelas ini (BCC, AKIEC, SCC, DF, VASC) tidak ada di ISIC 2017</t>
         </is>
@@ -3894,31 +3837,31 @@
           <t>ISIC 2019 Test</t>
         </is>
       </c>
-      <c r="B17" s="29" t="n">
+      <c r="B17" s="23" t="n">
         <v>374</v>
       </c>
-      <c r="C17" s="29" t="n">
+      <c r="C17" s="23" t="n">
         <v>975</v>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D17" s="23" t="n">
         <v>660</v>
       </c>
-      <c r="E17" s="29" t="n">
+      <c r="E17" s="23" t="n">
         <v>91</v>
       </c>
-      <c r="F17" s="29" t="n">
+      <c r="F17" s="23" t="n">
         <v>1327</v>
       </c>
-      <c r="G17" s="29" t="n">
+      <c r="G17" s="23" t="n">
         <v>2495</v>
       </c>
-      <c r="H17" s="29" t="n">
+      <c r="H17" s="23" t="n">
         <v>165</v>
       </c>
-      <c r="I17" s="29" t="n">
+      <c r="I17" s="23" t="n">
         <v>104</v>
       </c>
-      <c r="J17" s="29" t="n">
+      <c r="J17" s="23" t="n">
         <v>6191</v>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -3928,39 +3871,39 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="31" t="n">
+      <c r="B18" s="25" t="n">
         <v>1438</v>
       </c>
-      <c r="C18" s="31" t="n">
+      <c r="C18" s="25" t="n">
         <v>4298</v>
       </c>
-      <c r="D18" s="31" t="n">
+      <c r="D18" s="25" t="n">
         <v>660</v>
       </c>
-      <c r="E18" s="31" t="n">
+      <c r="E18" s="25" t="n">
         <v>330</v>
       </c>
-      <c r="F18" s="31" t="n">
+      <c r="F18" s="25" t="n">
         <v>1327</v>
       </c>
-      <c r="G18" s="31" t="n">
+      <c r="G18" s="25" t="n">
         <v>2495</v>
       </c>
-      <c r="H18" s="31" t="n">
+      <c r="H18" s="25" t="n">
         <v>596</v>
       </c>
-      <c r="I18" s="31" t="n">
+      <c r="I18" s="25" t="n">
         <v>357</v>
       </c>
-      <c r="J18" s="31" t="n">
+      <c r="J18" s="25" t="n">
         <v>11501</v>
       </c>
-      <c r="K18" s="26" t="inlineStr">
+      <c r="K18" s="20" t="inlineStr">
         <is>
           <t>11.501 + 22.051 = 33.552 (pas 100%)</t>
         </is>
@@ -3980,7 +3923,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00C0392B"/>
+    <tabColor rgb="00FF0000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -4011,17 +3954,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Daftar Lengkap Paper yang Dipakai</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -4061,40 +4004,40 @@
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="27" t="n">
+      <c r="A6" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Tschandl, P., Rosendahl, C., &amp; Kittler, H.</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="23" t="n">
         <v>2018</v>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>The HAM10000 dataset, a large collection of multi-source dermatoscopic images of common pigmented skin lesions</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Scientific Data, Vol. 5, Art. 180161</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Nature Research (Scopus Q1, IF: 9.8)</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Sumber utama dataset HAM10000 (10.015 citra) dan dasar resmi penggabungan Seborrheic Keratosis ke BKL.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="29" t="n">
+      <c r="A7" s="23" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -4102,7 +4045,7 @@
           <t>Codella, N. C. F., Gutman, D., Celebi, M. E., et al.</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="23" t="n">
         <v>2018</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -4127,40 +4070,40 @@
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="27" t="n">
+      <c r="A8" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Baig, A. R., Abbas, Q., Almakki, R., et al.</t>
         </is>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="23" t="n">
         <v>2023</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Light-Dermo: A lightweight pretrained convolution neural network for the diagnosis of multiclass skin lesions</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Diagnostics, Vol. 13, No. 3, Art. 385</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>MDPI (Scopus Q2, IF: 3.6)</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Rujukan penggabungan multi-dataset HAM10000 &amp; ISIC 2019 serta eliminasi duplikasi citra lesi.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="29" t="n">
+      <c r="A9" s="23" t="n">
         <v>4</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -4168,7 +4111,7 @@
           <t>Ichim, L., Mitrica, R. I., Serghei, M. O., &amp; Popescu, D.</t>
         </is>
       </c>
-      <c r="C9" s="29" t="n">
+      <c r="C9" s="23" t="n">
         <v>2023</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -4193,40 +4136,40 @@
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="27" t="n">
+      <c r="A10" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Barata, C., Celebi, M. E., &amp; Marques, J. S.</t>
         </is>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="23" t="n">
         <v>2020</v>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Explainable skin lesion diagnosis using taxonomies</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Pattern Recognition, Vol. 110, Art. 107413</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Elsevier (Scopus Q1, IF: 8.0)</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Rujukan pemetaan biner ISIC 2017: Melanoma = Ganas, Nevus &amp; Keratosis = Jinak.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="29" t="n">
+      <c r="A11" s="23" t="n">
         <v>6</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -4234,7 +4177,7 @@
           <t>Jojoa Acosta, M. F., Caballero Tovar, L. Y., et al.</t>
         </is>
       </c>
-      <c r="C11" s="29" t="n">
+      <c r="C11" s="23" t="n">
         <v>2021</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -4259,40 +4202,40 @@
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="27" t="n">
+      <c r="A12" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Kousis, I., Perikos, I., Hatzilygeroudis, I., &amp; Virvou, M.</t>
         </is>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="23" t="n">
         <v>2022</v>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Deep Learning Methods for Accurate Skin Cancer Recognition and Mobile Application</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Electronics, Vol. 11, No. 9, Art. 1294</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>MDPI (Scopus Q2, IF: 2.9)</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Konsensus biner HAM10000: NV, BKL, VASC, DF = Jinak; MEL, BCC, AKIEC = Ganas.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="29" t="n">
+      <c r="A13" s="23" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -4300,7 +4243,7 @@
           <t>Ghosh, P., Azam, S., Quadir, R., Karim, A., et al.</t>
         </is>
       </c>
-      <c r="C13" s="29" t="n">
+      <c r="C13" s="23" t="n">
         <v>2022</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -4325,40 +4268,40 @@
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="27" t="n">
+      <c r="A14" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Harangi, B., Baran, A., &amp; Hajdu, A.</t>
         </is>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="23" t="n">
         <v>2020</v>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Assisted deep learning framework for multi-class skin lesion classification considering a binary classification support</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Biomedical Signal Processing and Control, Vol. 62, Art. 102041</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Elsevier (Scopus Q1, IF: 5.1)</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Analisis transisi multiclass ke binary classification pada dataset ISIC 2018 / HAM10000.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="29" t="n">
+      <c r="A15" s="23" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -4366,7 +4309,7 @@
           <t>Yao, B., Jin, A., Liu, H., &amp; Li, Q.</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n">
+      <c r="C15" s="23" t="n">
         <v>2026</v>
       </c>
       <c r="D15" s="4" t="inlineStr">

</xml_diff>